<commit_message>
F3a: disarm-by-threshold fails for phasing checks (NaN CA50); track as-deployed warning XML
- 9049-openloop-audit.md: F3a live finding (2026-07-14, SimEnable) — CA50maxError
  at the 1e6 disarm sentinel still latches late-combustion: flat/no-combustion
  pressure makes the MFB normalization divide by ~0, CA50 goes NaN/Inf and beats
  any finite limit. Phasing checks need a validity guard, not a big threshold;
  non-finite sanitization is a systemic analytics gap (F8 family).
- parameter-files/CylWarningLevels.xml: as-retrieved from the 9049 (answers the
  'deployed warning-XML contents' open question).
- docs/cRIO9049 Warnings.xlsx: warning-limits worksheet update.
- .gitignore: flat_set/ (regenerable synthetic traces, same family as motored_set/).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/cRIO9049 Warnings.xlsx
+++ b/docs/cRIO9049 Warnings.xlsx
@@ -1,17 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RFSCtrlRoom\Desktop\Claude-Code-Projects\python-labview-controls-project\docs\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FBC95A7-CB2E-448D-98CA-C0A2BAA331AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Sheet1" sheetId="1" r:id="rId5"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="50">
   <si>
     <t>PC Label</t>
   </si>
@@ -28,6 +37,18 @@
     <t>Definition</t>
   </si>
   <si>
+    <t>Motoring Warning</t>
+  </si>
+  <si>
+    <t>Motoring Error</t>
+  </si>
+  <si>
+    <t>Fired Warning</t>
+  </si>
+  <si>
+    <t>Fired Error</t>
+  </si>
+  <si>
     <t>Maximum pressure</t>
   </si>
   <si>
@@ -40,6 +61,9 @@
     <t>MaxPCylMaxError</t>
   </si>
   <si>
+    <t>Per-cylinder peak pressure (Pmax) exceeds the limit; over-pressure protection. A latched error gates spark &amp; DI.</t>
+  </si>
+  <si>
     <t>Misfire 1 (self reg)</t>
   </si>
   <si>
@@ -49,42 +73,137 @@
     <t>MaxDevFromSelfAvgError</t>
   </si>
   <si>
+    <t>This cylinder's net IMEP deviates from its OWN running mean by more than the limit (per-cylinder cyclic misfire).</t>
+  </si>
+  <si>
     <t>Misfire 2 (cyl to cyl)</t>
   </si>
   <si>
+    <t>MaxDevFromAvgWarning</t>
+  </si>
+  <si>
+    <t>MaxDevFromAvgError</t>
+  </si>
+  <si>
+    <t>A cylinder's gross IMEP deviates from the across-cylinder average by more than the limit (one cylinder out of family).</t>
+  </si>
+  <si>
     <t>Misfire 3 (IMEPref)</t>
   </si>
   <si>
+    <t>MaxDevFromExpectedIMEPWarning</t>
+  </si>
+  <si>
+    <t>MaxDevFromExpectedIMEPError</t>
+  </si>
+  <si>
+    <t>Net IMEP deviates from the Expected-IMEP setpoint by more than the limit. NOTE: Expected IMEP is unwired (saved 0) as-built (audit F3) - disarm until it is actually driven.</t>
+  </si>
+  <si>
     <t>Cyclic variability</t>
   </si>
   <si>
+    <t>MaxIMEPstdWarning</t>
+  </si>
+  <si>
+    <t>MaxIMEPstdError</t>
+  </si>
+  <si>
+    <t>Running std-dev of net IMEP over the last N cycles exceeds the limit (N = 'samples for running IMEP std', default 20).</t>
+  </si>
+  <si>
     <t>MAPO</t>
   </si>
   <si>
+    <t>bar/CAD</t>
+  </si>
+  <si>
+    <t>MAPOmaxWarning</t>
+  </si>
+  <si>
+    <t>MAPOmaxError</t>
+  </si>
+  <si>
+    <t>Maximum Amplitude of Pressure Oscillation exceeds the limit (knock detection).</t>
+  </si>
+  <si>
+    <t>hand-set (knock data)</t>
+  </si>
+  <si>
     <t>Late combustion</t>
+  </si>
+  <si>
+    <t>CADATDC</t>
+  </si>
+  <si>
+    <t>CA50maxWarning</t>
+  </si>
+  <si>
+    <t>CA50maxError</t>
+  </si>
+  <si>
+    <t>CA50 (crank angle of 50% mass-fraction burned, deg ATDC) later than the limit (combustion phasing too retarded).</t>
+  </si>
+  <si>
+    <t>Notes:</t>
+  </si>
+  <si>
+    <t>• Provisional, synthetic-derived (real MONARCH geometry, NO engine run). Motoring = validated SIL-0 harness output (motored_set/); fired = synthetic --mode fired --q-fired 6000 set (fired_set/). Replace with real bench-motoring / light-off data.</t>
+  </si>
+  <si>
+    <t>• 1000000 = DISARMED (threshold so high it never trips) - metric meaningless in that mode (motoring has no combustion -&gt; CA50 / IMEPref / MAPO disarmed).</t>
+  </si>
+  <si>
+    <t>• MaxPCylMax Error = observed peak x1.3, UNCAPPED. Cap BOTH profiles at the engine's mechanical peak-cylinder-pressure rating when the team provides it (tune_thresholds --pmax-hard-limit &lt;rating&gt;).</t>
+  </si>
+  <si>
+    <t>• MaxDevFromExpectedIMEP (fired) REQUIRES 'Expected IMEP' actually driven (unwired/0 as-built, audit F3) - else disarm.</t>
+  </si>
+  <si>
+    <t>• MAPOmax (fired) = hand-set from knock-sensor/MAPO data (no MAPO column in the harness yet - see audit F3 / SIL-0 Step 4).</t>
+  </si>
+  <si>
+    <t>• Motoring std/dev rows (MaxIMEPstd, MaxDevFromAvg, MaxDevFromSelfAvg) sit at conservative FLOORS - synthetic cycles are identical (observed spread ~ 0); tighten from real motored data.</t>
+  </si>
+  <si>
+    <t>• 'samples for running IMEP std' = 20 (I32 window) - a separate config field, not a Warning/Error pair.</t>
+  </si>
+  <si>
+    <t>• Source: tools/tune_thresholds.py; workflow in docs/9049-openloop-audit.md §7 (SIL-0).</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="3">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="3">
@@ -92,7 +211,7 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -102,54 +221,64 @@
     </fill>
   </fills>
   <borders count="2">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
     <border>
       <left style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </left>
       <right style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </right>
       <top style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </top>
       <bottom style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+  <cellXfs count="6">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -339,114 +468,308 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:I18"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="19.0"/>
-    <col customWidth="1" min="2" max="2" width="7.38"/>
-    <col customWidth="1" min="3" max="3" width="23.5"/>
-    <col customWidth="1" min="4" max="4" width="22.25"/>
-    <col customWidth="1" min="5" max="5" width="42.63"/>
+    <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="2" max="2" width="9" customWidth="1"/>
+    <col min="3" max="3" width="30" customWidth="1"/>
+    <col min="4" max="4" width="28" customWidth="1"/>
+    <col min="5" max="5" width="147.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16" customWidth="1"/>
+    <col min="7" max="7" width="15" customWidth="1"/>
+    <col min="8" max="8" width="21.7109375" customWidth="1"/>
+    <col min="9" max="9" width="19.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="I1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="3"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="s">
+    </row>
+    <row r="2" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="3"/>
-      <c r="C3" s="2" t="s">
+      <c r="B2" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="C2" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="E3" s="3"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="s">
+      <c r="D2" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="s">
+      <c r="E2" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="s">
+      <c r="F2" s="5">
+        <v>181</v>
+      </c>
+      <c r="G2" s="5">
+        <v>196.1</v>
+      </c>
+      <c r="H2" s="5">
+        <v>213.5</v>
+      </c>
+      <c r="I2" s="5">
+        <v>231.3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="3"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="s">
+      <c r="B3" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="s">
+      <c r="D3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
+      <c r="E3" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" s="5">
+        <v>0.5</v>
+      </c>
+      <c r="G3" s="5">
+        <v>0.8</v>
+      </c>
+      <c r="H3" s="5">
+        <v>0.5</v>
+      </c>
+      <c r="I3" s="5">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4" s="5">
+        <v>0.5</v>
+      </c>
+      <c r="G4" s="5">
+        <v>0.8</v>
+      </c>
+      <c r="H4" s="5">
+        <v>0.5</v>
+      </c>
+      <c r="I4" s="5">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F5" s="5">
+        <v>1000000</v>
+      </c>
+      <c r="G5" s="5">
+        <v>1000000</v>
+      </c>
+      <c r="H5" s="5">
+        <v>10.33</v>
+      </c>
+      <c r="I5" s="5">
+        <v>15.5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="F6" s="5">
+        <v>0.2</v>
+      </c>
+      <c r="G6" s="5">
+        <v>0.3</v>
+      </c>
+      <c r="H6" s="5">
+        <v>0.2</v>
+      </c>
+      <c r="I6" s="5">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="F7" s="5">
+        <v>1000000</v>
+      </c>
+      <c r="G7" s="5">
+        <v>1000000</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="I7" s="5" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="F8" s="5">
+        <v>1000000</v>
+      </c>
+      <c r="G8" s="5">
+        <v>1000000</v>
+      </c>
+      <c r="H8" s="5">
+        <v>17.899999999999999</v>
+      </c>
+      <c r="I8" s="5">
+        <v>22.9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="2" t="s">
+        <v>49</v>
+      </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>